<commit_message>
project 3 - primary review
</commit_message>
<xml_diff>
--- a/backend/data/converted docs/SMS/PO04822-shipment-data.xlsx
+++ b/backend/data/converted docs/SMS/PO04822-shipment-data.xlsx
@@ -1,41 +1,149 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lam.le_tentree\Downloads\25026-p2-QuanLyHangDenKho-TuongLam-main\backend\data\converted docs\SMS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADC0205-15F3-44E9-9E42-9092990BBF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Shipment Data" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="39">
+  <si>
+    <t>CTN#</t>
+  </si>
+  <si>
+    <t>PO#</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>UPC</t>
+  </si>
+  <si>
+    <t>Knit/Woven</t>
+  </si>
+  <si>
+    <t>Style Description</t>
+  </si>
+  <si>
+    <t>Color Description</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Composition</t>
+  </si>
+  <si>
+    <t>HTS Code</t>
+  </si>
+  <si>
+    <t>Unit Price USD</t>
+  </si>
+  <si>
+    <t>Total USD</t>
+  </si>
+  <si>
+    <t>PCS/CTN</t>
+  </si>
+  <si>
+    <t>N/W (KGS)</t>
+  </si>
+  <si>
+    <t>G/W (KGS)</t>
+  </si>
+  <si>
+    <t>MEASURE (CM)</t>
+  </si>
+  <si>
+    <t>PO04822</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Knit</t>
+  </si>
+  <si>
+    <t>Freemont Henley</t>
+  </si>
+  <si>
+    <t>Slate Moss Heather</t>
+  </si>
+  <si>
+    <t>Henley</t>
+  </si>
+  <si>
+    <t>Men</t>
+  </si>
+  <si>
+    <t>58% Organic Cotton 39% Tencel 3% Elastane</t>
+  </si>
+  <si>
+    <t>61091000</t>
+  </si>
+  <si>
+    <t>50X35X20</t>
+  </si>
+  <si>
+    <t>Highwood Turtleneck</t>
+  </si>
+  <si>
+    <t>Willow Ash Heather</t>
+  </si>
+  <si>
+    <t>Top</t>
+  </si>
+  <si>
+    <t>Women</t>
+  </si>
+  <si>
+    <t>61046990</t>
+  </si>
+  <si>
+    <t>Steel Bay Heather</t>
+  </si>
+  <si>
+    <t>Sorrel Henley Longsleeve</t>
+  </si>
+  <si>
+    <t>ZCM5552-6933-M</t>
+  </si>
+  <si>
+    <t>ZCW5563-6902-S</t>
+  </si>
+  <si>
+    <t>ZCW5563-6942-S</t>
+  </si>
+  <si>
+    <t>ZCW7015-6902-S</t>
+  </si>
+  <si>
+    <t>ZCW7015-6942-S</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +173,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,95 +512,99 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>CTN#</v>
-      </c>
-      <c r="B1" t="str">
-        <v>PO#</v>
-      </c>
-      <c r="C1" t="str">
-        <v>SKU</v>
-      </c>
-      <c r="D1" t="str">
-        <v>UPC</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Knit/Woven</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Style Description</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Color Description</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Category</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Gender</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Composition</v>
-      </c>
-      <c r="K1" t="str">
-        <v>HTS Code</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Unit Price USD</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Total USD</v>
-      </c>
-      <c r="N1" t="str">
-        <v>PCS/CTN</v>
-      </c>
-      <c r="O1" t="str">
-        <v>N/W (KGS)</v>
-      </c>
-      <c r="P1" t="str">
-        <v>G/W (KGS)</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>MEASURE (CM)</v>
+    <row r="1" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
-        <v>PO04822</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ZCM5552-6933</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v>Knit</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Freemont Henley</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Slate Moss Heather</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Henley</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Men</v>
-      </c>
-      <c r="J2" t="str">
-        <v>58% Organic Cotton 39% Tencel 3% Elastane</v>
-      </c>
-      <c r="K2" t="str">
-        <v>61091000</v>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
       </c>
       <c r="L2">
         <v>14.99</v>
@@ -501,43 +621,43 @@
       <c r="P2">
         <v>7.3</v>
       </c>
-      <c r="Q2" t="str">
-        <v>50X35X20</v>
+      <c r="Q2" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="str">
-        <v>PO04822</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ZCW5563-6902</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>Knit</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Highwood Turtleneck</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Willow Ash Heather</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Top</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Women</v>
-      </c>
-      <c r="J3" t="str">
-        <v>58% Organic Cotton 39% Tencel 3% Elastane</v>
-      </c>
-      <c r="K3" t="str">
-        <v>61046990</v>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
       </c>
       <c r="L3">
         <v>14.64</v>
@@ -548,49 +668,49 @@
       <c r="N3">
         <v>1</v>
       </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
+      <c r="O3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" t="str">
-        <v>PO04822</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ZCW5563-6942</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v>Knit</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Highwood Turtleneck</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Steel Bay Heather</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Top</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Women</v>
-      </c>
-      <c r="J4" t="str">
-        <v>58% Organic Cotton 39% Tencel 3% Elastane</v>
-      </c>
-      <c r="K4" t="str">
-        <v>61046990</v>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
       </c>
       <c r="L4">
         <v>14.64</v>
@@ -601,49 +721,49 @@
       <c r="N4">
         <v>7</v>
       </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
+      <c r="O4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" t="str">
-        <v>PO04822</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ZCW7015-6902</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v>Knit</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Sorrel Henley Longsleeve</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Willow Ash Heather</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Top</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Women</v>
-      </c>
-      <c r="J5" t="str">
-        <v>58% Organic Cotton 39% Tencel 3% Elastane</v>
-      </c>
-      <c r="K5" t="str">
-        <v>61046990</v>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="s">
+        <v>31</v>
       </c>
       <c r="L5">
         <v>6.38</v>
@@ -654,49 +774,49 @@
       <c r="N5">
         <v>7</v>
       </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
-        <v/>
+      <c r="O5" t="s">
+        <v>18</v>
+      </c>
+      <c r="P5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
-      <c r="B6" t="str">
-        <v>PO04822</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ZCW7015-6942</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v>Knit</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Sorrel Henley Longsleeve</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Steel Bay Heather</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Top</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Women</v>
-      </c>
-      <c r="J6" t="str">
-        <v>58% Organic Cotton 39% Tencel 3% Elastane</v>
-      </c>
-      <c r="K6" t="str">
-        <v>61046990</v>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" t="s">
+        <v>31</v>
       </c>
       <c r="L6">
         <v>6.38</v>
@@ -707,19 +827,20 @@
       <c r="N6">
         <v>1</v>
       </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v/>
+      <c r="O6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q6"/>
+    <ignoredError sqref="A1:Q1 A6:B6 A2:B2 D2:Q2 A3:B3 D3:Q3 A4:B4 D4:Q4 A5:B5 D5:Q5 D6:Q6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>